<commit_message>
docs(tutorials): FEM-3 — the reader states the toe: Tip = pinned on the shafts and the wall before the first run; completed wall file carries pinned
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_pile_wall.xlsx
+++ b/docs/tutorials/files/xslope_pile_wall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1F2F76-FB33-0143-929F-736B2B93C722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE192E0-97C6-CB43-9291-6C4E11A86E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="317">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1128,6 +1128,9 @@
   </si>
   <si>
     <t>Tip</t>
+  </si>
+  <si>
+    <t>Pinned</t>
   </si>
 </sst>
 </file>
@@ -4180,11 +4183,11 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>pinned</t>
         </is>
       </c>
       <c r="Z3" t="s">
-        <v>226</v>
+        <v>316</v>
       </c>
       <c r="AA3" t="s">
         <v>263</v>
@@ -4210,6 +4213,9 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
+      <c r="Z4" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
@@ -4403,11 +4409,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
-      <formula1>$Z$2:$Z$3</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H12" xr:uid="{00000000-0002-0000-0A00-000001000000}">
       <formula1>$AA$2:$AA$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+      <formula1>$Z$2:$Z$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9533,6 +9539,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -9549,20 +9569,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10929,6 +10935,23 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH4:AI4"/>
@@ -10942,23 +10965,6 @@
     <mergeCell ref="AN7:AO7"/>
     <mergeCell ref="AH7:AI7"/>
     <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">

</xml_diff>

<commit_message>
tutorial(fem03): the wall tutorial's two models declare t_cut = 0
The bare slope and the completed wall model left the tensile cutoff blank on
their one Mohr-Coulomb row, so Run FEM raised the unbounded-tension warning on
both and the clay was free to carry tension up to c/tan(phi) = 549.5 psf under
the wall's bending. Each now declares t_cut = 0 on the soil row.

Written through xslope.fileio.write_cells_to_xlsx; the cell-level diff on each
workbook is mat!L11 and nothing else, and load_slope_data reads 0.0 back.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_pile_wall.xlsx
+++ b/docs/tutorials/files/xslope_pile_wall.xlsx
@@ -6768,7 +6768,9 @@
       <c r="K11" s="3">
         <v>0.0</v>
       </c>
-      <c r="L11" s="3"/>
+      <c r="L11" s="3">
+        <v>0</v>
+      </c>
       <c r="M11" s="3">
         <v>2000000.0</v>
       </c>

</xml_diff>